<commit_message>
Add Amazon Reconciliation tab + collapse Amazon rules to one regex
- Rules!A43: replace fragile per-transaction Amazon patterns with a single
  case-insensitive regex (AMZN|AMAZON). Refund rule (row 19) unchanged and
  stays above it (first-match-wins), so refunds still book as income.
- New 'Amazon Reconciliation' tab: pulls the monthly Amazon total from
  CC Detail row 14, lets you split it into real categories (with a
  red flag when a month isn't fully reconciled), shows 'true' category
  totals (native + Amazon), and lists live Amazon transactions via FILTER
  as a splitting aid. No Apps Script changes required.
</commit_message>
<xml_diff>
--- a/Family_Income_Statement_2026_v5_FIRE.xlsx
+++ b/Family_Income_Statement_2026_v5_FIRE.xlsx
@@ -17,6 +17,7 @@
     <sheet name="Rules" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="Pension - Sue" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="FIRE Dashboard" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Amazon Reconciliation" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -244,7 +245,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -395,11 +396,18 @@
     <xf numFmtId="0" fontId="15" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="11" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="16" fillId="13" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="10" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="16" fillId="11" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
     <dxf>
       <font>
         <b val="1"/>
@@ -419,6 +427,16 @@
         <patternFill/>
       </fill>
       <border/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="009C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <colors>
@@ -12814,12 +12832,17 @@
     <row r="43" ht="15.75" customHeight="1" s="39">
       <c r="A43" s="38" t="inlineStr">
         <is>
-          <t>AMAZON MKTPL|AMZN|Amazon.com*RT85D8PV3|AMAZON PRIME*B40RT9363</t>
+          <t>AMZN|AMAZON</t>
         </is>
       </c>
       <c r="B43" s="38" t="inlineStr">
         <is>
           <t>Amazon (misc)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Catch-all Amazon → reconcile on 'Amazon Reconciliation' tab</t>
         </is>
       </c>
     </row>
@@ -15536,6 +15559,969 @@
     <mergeCell ref="A69:C70"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00BF8F00"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" style="39" min="1" max="1"/>
+    <col width="34" customWidth="1" style="39" min="2" max="2"/>
+    <col width="9" customWidth="1" style="39" min="3" max="3"/>
+    <col width="9" customWidth="1" style="39" min="4" max="4"/>
+    <col width="9" customWidth="1" style="39" min="5" max="5"/>
+    <col width="9" customWidth="1" style="39" min="6" max="6"/>
+    <col width="9" customWidth="1" style="39" min="7" max="7"/>
+    <col width="9" customWidth="1" style="39" min="8" max="8"/>
+    <col width="9" customWidth="1" style="39" min="9" max="9"/>
+    <col width="9" customWidth="1" style="39" min="10" max="10"/>
+    <col width="9" customWidth="1" style="39" min="11" max="11"/>
+    <col width="9" customWidth="1" style="39" min="12" max="12"/>
+    <col width="9" customWidth="1" style="39" min="13" max="13"/>
+    <col width="11" customWidth="1" style="39" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="40" t="inlineStr">
+        <is>
+          <t>Amazon — Monthly Reconciliation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1" s="39">
+      <c r="A2" s="41" t="inlineStr">
+        <is>
+          <t>All Amazon spend now lands in ONE bucket — 'Amazon (misc)', CC Detail row 14 — via a single regex rule (AMZN|AMAZON). Each month, split that total into real categories below. ORANGE = you enter $. The reference list at the bottom shows the actual Amazon transactions to guide the split.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="42" t="inlineStr">
+        <is>
+          <t>① AMAZON TOTAL TO RECONCILE  (auto — from CC Detail)</t>
+        </is>
+      </c>
+      <c r="B4" s="43" t="n"/>
+      <c r="C4" s="43" t="n"/>
+      <c r="D4" s="43" t="n"/>
+      <c r="E4" s="43" t="n"/>
+      <c r="F4" s="43" t="n"/>
+      <c r="G4" s="43" t="n"/>
+      <c r="H4" s="43" t="n"/>
+      <c r="I4" s="43" t="n"/>
+      <c r="J4" s="43" t="n"/>
+      <c r="K4" s="43" t="n"/>
+      <c r="L4" s="43" t="n"/>
+      <c r="M4" s="43" t="n"/>
+      <c r="N4" s="43" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="78" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B5" s="51" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="C5" s="51" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="D5" s="51" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="E5" s="51" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="F5" s="51" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="G5" s="51" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="H5" s="51" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="I5" s="51" t="inlineStr">
+        <is>
+          <t>Aug</t>
+        </is>
+      </c>
+      <c r="J5" s="51" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="K5" s="51" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="L5" s="51" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="M5" s="51" t="inlineStr">
+        <is>
+          <t>Dec</t>
+        </is>
+      </c>
+      <c r="N5" s="51" t="inlineStr">
+        <is>
+          <t>YTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="79" t="inlineStr">
+        <is>
+          <t>Amazon (misc) — to reconcile</t>
+        </is>
+      </c>
+      <c r="B6" s="80">
+        <f>'CC Detail'!B14</f>
+        <v/>
+      </c>
+      <c r="C6" s="80">
+        <f>'CC Detail'!C14</f>
+        <v/>
+      </c>
+      <c r="D6" s="80">
+        <f>'CC Detail'!D14</f>
+        <v/>
+      </c>
+      <c r="E6" s="80">
+        <f>'CC Detail'!E14</f>
+        <v/>
+      </c>
+      <c r="F6" s="80">
+        <f>'CC Detail'!F14</f>
+        <v/>
+      </c>
+      <c r="G6" s="80">
+        <f>'CC Detail'!G14</f>
+        <v/>
+      </c>
+      <c r="H6" s="80">
+        <f>'CC Detail'!H14</f>
+        <v/>
+      </c>
+      <c r="I6" s="80">
+        <f>'CC Detail'!I14</f>
+        <v/>
+      </c>
+      <c r="J6" s="80">
+        <f>'CC Detail'!J14</f>
+        <v/>
+      </c>
+      <c r="K6" s="80">
+        <f>'CC Detail'!K14</f>
+        <v/>
+      </c>
+      <c r="L6" s="80">
+        <f>'CC Detail'!L14</f>
+        <v/>
+      </c>
+      <c r="M6" s="80">
+        <f>'CC Detail'!M14</f>
+        <v/>
+      </c>
+      <c r="N6" s="81">
+        <f>SUM(B6:M6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="42" t="inlineStr">
+        <is>
+          <t>② ALLOCATE INTO CATEGORIES  (enter $ per month)</t>
+        </is>
+      </c>
+      <c r="B8" s="43" t="n"/>
+      <c r="C8" s="43" t="n"/>
+      <c r="D8" s="43" t="n"/>
+      <c r="E8" s="43" t="n"/>
+      <c r="F8" s="43" t="n"/>
+      <c r="G8" s="43" t="n"/>
+      <c r="H8" s="43" t="n"/>
+      <c r="I8" s="43" t="n"/>
+      <c r="J8" s="43" t="n"/>
+      <c r="K8" s="43" t="n"/>
+      <c r="L8" s="43" t="n"/>
+      <c r="M8" s="43" t="n"/>
+      <c r="N8" s="43" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="78" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B9" s="51" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="C9" s="51" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="D9" s="51" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="E9" s="51" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="F9" s="51" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="G9" s="51" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="H9" s="51" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="I9" s="51" t="inlineStr">
+        <is>
+          <t>Aug</t>
+        </is>
+      </c>
+      <c r="J9" s="51" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="K9" s="51" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="L9" s="51" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="M9" s="51" t="inlineStr">
+        <is>
+          <t>Dec</t>
+        </is>
+      </c>
+      <c r="N9" s="51" t="inlineStr">
+        <is>
+          <t>YTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="82" t="inlineStr">
+        <is>
+          <t>Groceries</t>
+        </is>
+      </c>
+      <c r="B10" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="80">
+        <f>SUM(B10:M10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="82" t="inlineStr">
+        <is>
+          <t>Kids / Activities</t>
+        </is>
+      </c>
+      <c r="B11" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="80">
+        <f>SUM(B11:M11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="82" t="inlineStr">
+        <is>
+          <t>Personal Care</t>
+        </is>
+      </c>
+      <c r="B12" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="80">
+        <f>SUM(B12:M12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="82" t="inlineStr">
+        <is>
+          <t>Pharmacy / Health</t>
+        </is>
+      </c>
+      <c r="B13" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="80">
+        <f>SUM(B13:M13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="82" t="inlineStr">
+        <is>
+          <t>Home / Hardware</t>
+        </is>
+      </c>
+      <c r="B14" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="80">
+        <f>SUM(B14:M14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="82" t="inlineStr">
+        <is>
+          <t>Subscriptions (Prime/Kindle/Audible)</t>
+        </is>
+      </c>
+      <c r="B15" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="80">
+        <f>SUM(B15:M15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="82" t="inlineStr">
+        <is>
+          <t>Other / gifts</t>
+        </is>
+      </c>
+      <c r="B16" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="83" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="80">
+        <f>SUM(B16:M16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="79" t="inlineStr">
+        <is>
+          <t>Allocated total</t>
+        </is>
+      </c>
+      <c r="B17" s="84">
+        <f>SUM(B10:B16)</f>
+        <v/>
+      </c>
+      <c r="C17" s="84">
+        <f>SUM(C10:C16)</f>
+        <v/>
+      </c>
+      <c r="D17" s="84">
+        <f>SUM(D10:D16)</f>
+        <v/>
+      </c>
+      <c r="E17" s="84">
+        <f>SUM(E10:E16)</f>
+        <v/>
+      </c>
+      <c r="F17" s="84">
+        <f>SUM(F10:F16)</f>
+        <v/>
+      </c>
+      <c r="G17" s="84">
+        <f>SUM(G10:G16)</f>
+        <v/>
+      </c>
+      <c r="H17" s="84">
+        <f>SUM(H10:H16)</f>
+        <v/>
+      </c>
+      <c r="I17" s="84">
+        <f>SUM(I10:I16)</f>
+        <v/>
+      </c>
+      <c r="J17" s="84">
+        <f>SUM(J10:J16)</f>
+        <v/>
+      </c>
+      <c r="K17" s="84">
+        <f>SUM(K10:K16)</f>
+        <v/>
+      </c>
+      <c r="L17" s="84">
+        <f>SUM(L10:L16)</f>
+        <v/>
+      </c>
+      <c r="M17" s="84">
+        <f>SUM(M10:M16)</f>
+        <v/>
+      </c>
+      <c r="N17" s="84">
+        <f>SUM(N10:N16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="79" t="inlineStr">
+        <is>
+          <t>Unallocated remaining</t>
+        </is>
+      </c>
+      <c r="B18" s="81">
+        <f>B6-B17</f>
+        <v/>
+      </c>
+      <c r="C18" s="81">
+        <f>C6-C17</f>
+        <v/>
+      </c>
+      <c r="D18" s="81">
+        <f>D6-D17</f>
+        <v/>
+      </c>
+      <c r="E18" s="81">
+        <f>E6-E17</f>
+        <v/>
+      </c>
+      <c r="F18" s="81">
+        <f>F6-F17</f>
+        <v/>
+      </c>
+      <c r="G18" s="81">
+        <f>G6-G17</f>
+        <v/>
+      </c>
+      <c r="H18" s="81">
+        <f>H6-H17</f>
+        <v/>
+      </c>
+      <c r="I18" s="81">
+        <f>I6-I17</f>
+        <v/>
+      </c>
+      <c r="J18" s="81">
+        <f>J6-J17</f>
+        <v/>
+      </c>
+      <c r="K18" s="81">
+        <f>K6-K17</f>
+        <v/>
+      </c>
+      <c r="L18" s="81">
+        <f>L6-L17</f>
+        <v/>
+      </c>
+      <c r="M18" s="81">
+        <f>M6-M17</f>
+        <v/>
+      </c>
+      <c r="N18" s="81">
+        <f>N6-N17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="42" t="inlineStr">
+        <is>
+          <t>③ RECONCILED CATEGORY TOTALS (YTD) — the un-muddied picture</t>
+        </is>
+      </c>
+      <c r="B20" s="43" t="n"/>
+      <c r="C20" s="43" t="n"/>
+      <c r="D20" s="43" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="78" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B21" s="51" t="inlineStr">
+        <is>
+          <t>Native (CC Detail)</t>
+        </is>
+      </c>
+      <c r="C21" s="51" t="inlineStr">
+        <is>
+          <t>+ Amazon</t>
+        </is>
+      </c>
+      <c r="D21" s="51">
+        <f> True total (YTD)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="82" t="inlineStr">
+        <is>
+          <t>Groceries</t>
+        </is>
+      </c>
+      <c r="B22" s="80">
+        <f>'CC Detail'!N5</f>
+        <v/>
+      </c>
+      <c r="C22" s="80">
+        <f>N10</f>
+        <v/>
+      </c>
+      <c r="D22" s="81">
+        <f>B22+C22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="82" t="inlineStr">
+        <is>
+          <t>Kids / Activities</t>
+        </is>
+      </c>
+      <c r="B23" s="80">
+        <f>'CC Detail'!N9</f>
+        <v/>
+      </c>
+      <c r="C23" s="80">
+        <f>N11</f>
+        <v/>
+      </c>
+      <c r="D23" s="81">
+        <f>B23+C23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="82" t="inlineStr">
+        <is>
+          <t>Personal Care</t>
+        </is>
+      </c>
+      <c r="B24" s="80">
+        <f>'CC Detail'!N11</f>
+        <v/>
+      </c>
+      <c r="C24" s="80">
+        <f>N12</f>
+        <v/>
+      </c>
+      <c r="D24" s="81">
+        <f>B24+C24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="82" t="inlineStr">
+        <is>
+          <t>Pharmacy / Health</t>
+        </is>
+      </c>
+      <c r="B25" s="80">
+        <f>'CC Detail'!N12</f>
+        <v/>
+      </c>
+      <c r="C25" s="80">
+        <f>N13</f>
+        <v/>
+      </c>
+      <c r="D25" s="81">
+        <f>B25+C25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="82" t="inlineStr">
+        <is>
+          <t>Home / Hardware</t>
+        </is>
+      </c>
+      <c r="B26" s="80">
+        <f>'CC Detail'!N13</f>
+        <v/>
+      </c>
+      <c r="C26" s="80">
+        <f>N14</f>
+        <v/>
+      </c>
+      <c r="D26" s="81">
+        <f>B26+C26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="82" t="inlineStr">
+        <is>
+          <t>Subscriptions</t>
+        </is>
+      </c>
+      <c r="B27" s="80">
+        <f>'CC Detail'!N8</f>
+        <v/>
+      </c>
+      <c r="C27" s="80">
+        <f>N15</f>
+        <v/>
+      </c>
+      <c r="D27" s="81">
+        <f>B27+C27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="82" t="inlineStr">
+        <is>
+          <t>Other / gifts</t>
+        </is>
+      </c>
+      <c r="B28" s="80">
+        <f>'CC Detail'!N17</f>
+        <v/>
+      </c>
+      <c r="C28" s="80">
+        <f>N16</f>
+        <v/>
+      </c>
+      <c r="D28" s="81">
+        <f>B28+C28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="68" t="inlineStr">
+        <is>
+          <t>Note: once split, these 'true totals' show real spend per category — Amazon no longer hides hardware, hygiene, and kids' purchases in one lump. Feed these into the guardrail when it's built.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
+    <row r="32">
+      <c r="A32" s="42" t="inlineStr">
+        <is>
+          <t>④ REFERENCE — current Amazon transactions  (auto, read-only)</t>
+        </is>
+      </c>
+      <c r="B32" s="43" t="n"/>
+      <c r="C32" s="43" t="n"/>
+      <c r="D32" s="43" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="68" t="inlineStr">
+        <is>
+          <t>Pulls Amazon rows from your Barclay import so you can see what to split. Refreshes when you paste new data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="78" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B34" s="78" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C34" s="51" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="D34" s="51" t="inlineStr">
+        <is>
+          <t>Purchased by</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35">
+        <f>IFERROR(FILTER({'Imports - Barclay'!A5:A,'Imports - Barclay'!B5:B,'Imports - Barclay'!D5:D,'Imports - Barclay'!F5:F},REGEXMATCH(UPPER('Imports - Barclay'!B5:B),"AMZN|AMAZON")),"No Amazon rows in current Barclay import")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A29:D30"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A33:D33"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B18:N18">
+    <cfRule type="cellIs" priority="1" operator="notBetween" dxfId="2">
+      <formula>-1</formula>
+      <formula>1</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add guided Monthly Entry tab + Apps Script distributor and optional Google Form
- 'Monthly Entry' tab: one guided worksheet with a month dropdown and
  sections for Balances, Solar energy, electric bill, Amazon split, and
  Comp & Benefits YTD. Pulls the month's Amazon total for reference.
- apps_script/MonthlyEntry.gs:
  * postMonthlyEntry() fans staged values out to the correct cell/column
    across all destination tabs for the chosen month (blanks skipped,
    with a confirmation dialog and an auditable MAP).
  * createMonthlyForm() builds a linked Google Form; onMonthlyFormSubmit()
    funnels responses into the Monthly Entry tab and auto-distributes.
  * clearMonthlyEntry() resets inputs for the next month.
</commit_message>
<xml_diff>
--- a/Family_Income_Statement_2026_v5_FIRE.xlsx
+++ b/Family_Income_Statement_2026_v5_FIRE.xlsx
@@ -20,6 +20,7 @@
     <sheet name="Amazon Reconciliation" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="Solar Reinvestment" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="HSA Election Planner" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Monthly Entry" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -248,7 +249,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -417,6 +418,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -18371,6 +18373,494 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="007030A0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C52"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" style="39" min="1" max="1"/>
+    <col width="14" customWidth="1" style="39" min="2" max="2"/>
+    <col width="46" customWidth="1" style="39" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="42" t="inlineStr">
+        <is>
+          <t>Monthly Entry — one place to update everything</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1" s="39">
+      <c r="A2" s="43" t="inlineStr">
+        <is>
+          <t>Pick the month, fill in what you have (blanks are skipped), then run 📊 Family Finances → Post Monthly Entry. Values fan out to Balances, Solar, Amazon Reconciliation and Comp &amp; Benefits. You can also fill this from your phone via the linked Google Form.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="63" t="inlineStr">
+        <is>
+          <t>Month to post</t>
+        </is>
+      </c>
+      <c r="B4" s="49" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="C4" s="47" t="inlineStr">
+        <is>
+          <t>Choose the month these figures belong to.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Data as of (date)</t>
+        </is>
+      </c>
+      <c r="B5" s="94" t="n"/>
+      <c r="C5" s="47" t="inlineStr">
+        <is>
+          <t>Optional — for your records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="44" t="inlineStr">
+        <is>
+          <t>① ACCOUNT BALANCES  (month-end)</t>
+        </is>
+      </c>
+      <c r="B6" s="45" t="n"/>
+      <c r="C6" s="45" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Capital One Checking</t>
+        </is>
+      </c>
+      <c r="B7" s="50" t="n"/>
+      <c r="C7" s="47" t="inlineStr">
+        <is>
+          <t>→ Balances</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Capital One Savings</t>
+        </is>
+      </c>
+      <c r="B8" s="50" t="n"/>
+      <c r="C8" s="47" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Venmo float</t>
+        </is>
+      </c>
+      <c r="B9" s="50" t="n"/>
+      <c r="C9" s="47" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Fidelity Money Market</t>
+        </is>
+      </c>
+      <c r="B10" s="50" t="n"/>
+      <c r="C10" s="47" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Schwab investment</t>
+        </is>
+      </c>
+      <c r="B11" s="50" t="n"/>
+      <c r="C11" s="47" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>529</t>
+        </is>
+      </c>
+      <c r="B12" s="50" t="n"/>
+      <c r="C12" s="47" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>FSA Dep Care balance</t>
+        </is>
+      </c>
+      <c r="B13" s="50" t="n"/>
+      <c r="C13" s="47" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>FSA Health Care balance</t>
+        </is>
+      </c>
+      <c r="B14" s="50" t="n"/>
+      <c r="C14" s="47" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Matt 401k</t>
+        </is>
+      </c>
+      <c r="B15" s="50" t="n"/>
+      <c r="C15" s="47" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Sue 403b</t>
+        </is>
+      </c>
+      <c r="B16" s="50" t="n"/>
+      <c r="C16" s="47" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Sue pension (est.)</t>
+        </is>
+      </c>
+      <c r="B17" s="50" t="n"/>
+      <c r="C17" s="47" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B18" s="50" t="n"/>
+      <c r="C18" s="47" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="44" t="inlineStr">
+        <is>
+          <t>② SOLAR — ENERGY  (Enphase, kWh)</t>
+        </is>
+      </c>
+      <c r="B20" s="45" t="n"/>
+      <c r="C20" s="45" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Produced (kWh)</t>
+        </is>
+      </c>
+      <c r="B21" s="91" t="n"/>
+      <c r="C21" s="47" t="inlineStr">
+        <is>
+          <t>→ Solar Reinvestment log</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Consumed (kWh)</t>
+        </is>
+      </c>
+      <c r="B22" s="91" t="n"/>
+      <c r="C22" s="47" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Imported (kWh)</t>
+        </is>
+      </c>
+      <c r="B23" s="91" t="n"/>
+      <c r="C23" s="47" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Exported (kWh)</t>
+        </is>
+      </c>
+      <c r="B24" s="91" t="n"/>
+      <c r="C24" s="47" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="44" t="inlineStr">
+        <is>
+          <t>③ SOLAR — ELECTRIC BILL</t>
+        </is>
+      </c>
+      <c r="B25" s="45" t="n"/>
+      <c r="C25" s="45" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Baseline electric (would-have-paid)</t>
+        </is>
+      </c>
+      <c r="B26" s="50" t="n"/>
+      <c r="C26" s="47" t="inlineStr">
+        <is>
+          <t>→ Solar ROI row 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Actual electric bill</t>
+        </is>
+      </c>
+      <c r="B27" s="50" t="n"/>
+      <c r="C27" s="47" t="inlineStr">
+        <is>
+          <t>→ Solar ROI row 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="44" t="inlineStr">
+        <is>
+          <t>④ AMAZON — split this month's total into buckets</t>
+        </is>
+      </c>
+      <c r="B29" s="45" t="n"/>
+      <c r="C29" s="45" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Amazon total to split (auto)</t>
+        </is>
+      </c>
+      <c r="B30" s="73">
+        <f>IFERROR(INDEX('CC Detail'!B14:M14,MATCH($B$4,{"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec"},0)),"")</f>
+        <v/>
+      </c>
+      <c r="C30" s="47" t="inlineStr">
+        <is>
+          <t>Pulled from CC Detail for the chosen month — split it below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Groceries</t>
+        </is>
+      </c>
+      <c r="B31" s="50" t="n"/>
+      <c r="C31" s="47" t="inlineStr">
+        <is>
+          <t>→ Amazon Reconciliation</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Kids / Activities</t>
+        </is>
+      </c>
+      <c r="B32" s="50" t="n"/>
+      <c r="C32" s="47" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Personal Care</t>
+        </is>
+      </c>
+      <c r="B33" s="50" t="n"/>
+      <c r="C33" s="47" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Pharmacy / Health</t>
+        </is>
+      </c>
+      <c r="B34" s="50" t="n"/>
+      <c r="C34" s="47" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Home / Hardware</t>
+        </is>
+      </c>
+      <c r="B35" s="50" t="n"/>
+      <c r="C35" s="47" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Subscriptions</t>
+        </is>
+      </c>
+      <c r="B36" s="50" t="n"/>
+      <c r="C36" s="47" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Other / gifts</t>
+        </is>
+      </c>
+      <c r="B37" s="50" t="n"/>
+      <c r="C37" s="47" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Split check (should match total)</t>
+        </is>
+      </c>
+      <c r="B38" s="73">
+        <f>SUM(B31:B37)</f>
+        <v/>
+      </c>
+      <c r="C38" s="47" t="inlineStr">
+        <is>
+          <t>Compare to Amazon total above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="44" t="inlineStr">
+        <is>
+          <t>⑤ COMP &amp; BENEFITS  (YTD, from paystub)</t>
+        </is>
+      </c>
+      <c r="B40" s="45" t="n"/>
+      <c r="C40" s="45" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Matt gross earnings YTD</t>
+        </is>
+      </c>
+      <c r="B41" s="50" t="n"/>
+      <c r="C41" s="47" t="inlineStr">
+        <is>
+          <t>→ Comp &amp; Benefits</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Matt 401k contribution YTD</t>
+        </is>
+      </c>
+      <c r="B42" s="50" t="n"/>
+      <c r="C42" s="47" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Matt 401k match YTD</t>
+        </is>
+      </c>
+      <c r="B43" s="50" t="n"/>
+      <c r="C43" s="47" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>FSA Dep Care YTD</t>
+        </is>
+      </c>
+      <c r="B44" s="50" t="n"/>
+      <c r="C44" s="47" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>FSA Health Care YTD</t>
+        </is>
+      </c>
+      <c r="B45" s="50" t="n"/>
+      <c r="C45" s="47" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Tuition reimbursement YTD</t>
+        </is>
+      </c>
+      <c r="B46" s="50" t="n"/>
+      <c r="C46" s="47" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Stakeholder earnings YTD</t>
+        </is>
+      </c>
+      <c r="B47" s="50" t="n"/>
+      <c r="C47" s="47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Sue 403b YTD</t>
+        </is>
+      </c>
+      <c r="B48" s="50" t="n"/>
+      <c r="C48" s="47" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>529 contributions YTD</t>
+        </is>
+      </c>
+      <c r="B49" s="50" t="n"/>
+      <c r="C49" s="47" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="41" t="inlineStr">
+        <is>
+          <t>After posting, blank the input cells for next month (or use the Form). The script only writes fields you filled, into the month you chose above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A51:C52"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Jan,Feb,Mar,Apr,May,Jun,Jul,Aug,Sep,Oct,Nov,Dec"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add three-lane Spending Guardrail with rollover; wire actuals into Monthly Entry
- 'Spending Guardrail' tab: Matt / Sue / Household lanes ($200/$200/$300
  default), monthly tracker where unused budget ROLLS OVER. Standings panel
  shows each lane's rollover balance for a chosen month with a verdict
  (over-pause / on-track / splurge-OK), red/green conditional formatting,
  and a 'compounded cost of overspend' figure linked to the FIRE real return.
- Monthly Entry: added three discretionary-spend fields (Matt/Sue/Household)
  that post to the guardrail's actual rows for the chosen month.
- MonthlyEntry.gs: extended the distributor MAP and the Google Form + FORM_MAP
  to include the discretionary fields.
</commit_message>
<xml_diff>
--- a/Family_Income_Statement_2026_v5_FIRE.xlsx
+++ b/Family_Income_Statement_2026_v5_FIRE.xlsx
@@ -21,6 +21,7 @@
     <sheet name="Solar Reinvestment" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="HSA Election Planner" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="Monthly Entry" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Spending Guardrail" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -249,7 +250,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -419,11 +420,14 @@
     </xf>
     <xf numFmtId="166" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="16" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
     <dxf>
       <font>
         <b val="1"/>
@@ -451,6 +455,16 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -18380,7 +18394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" style="39" min="1" max="1"/>
@@ -18840,20 +18854,1170 @@
       <c r="C49" s="47" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="41" t="inlineStr">
+      <c r="A51" s="44" t="inlineStr">
+        <is>
+          <t>⑥ DISCRETIONARY SPENT  (this month)</t>
+        </is>
+      </c>
+      <c r="B51" s="45" t="n"/>
+      <c r="C51" s="45" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Matt discretionary spent</t>
+        </is>
+      </c>
+      <c r="B52" s="50" t="n"/>
+      <c r="C52" s="47" t="inlineStr">
+        <is>
+          <t>→ Spending Guardrail</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Sue discretionary spent</t>
+        </is>
+      </c>
+      <c r="B53" s="50" t="n"/>
+      <c r="C53" s="47" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Household discretionary spent</t>
+        </is>
+      </c>
+      <c r="B54" s="50" t="n"/>
+      <c r="C54" s="47" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="41" t="inlineStr">
         <is>
           <t>After posting, blank the input cells for next month (or use the Form). The script only writes fields you filled, into the month you chose above.</t>
         </is>
       </c>
     </row>
-    <row r="52"/>
+    <row r="57"/>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A51:C52"/>
+    <mergeCell ref="A56:C57"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Jan,Feb,Mar,Apr,May,Jun,Jul,Aug,Sep,Oct,Nov,Dec"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00C00000"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" style="39" min="1" max="1"/>
+    <col width="8" customWidth="1" style="39" min="2" max="2"/>
+    <col width="8" customWidth="1" style="39" min="3" max="3"/>
+    <col width="8" customWidth="1" style="39" min="4" max="4"/>
+    <col width="8" customWidth="1" style="39" min="5" max="5"/>
+    <col width="8" customWidth="1" style="39" min="6" max="6"/>
+    <col width="8" customWidth="1" style="39" min="7" max="7"/>
+    <col width="8" customWidth="1" style="39" min="8" max="8"/>
+    <col width="8" customWidth="1" style="39" min="9" max="9"/>
+    <col width="8" customWidth="1" style="39" min="10" max="10"/>
+    <col width="8" customWidth="1" style="39" min="11" max="11"/>
+    <col width="8" customWidth="1" style="39" min="12" max="12"/>
+    <col width="8" customWidth="1" style="39" min="13" max="13"/>
+    <col width="10" customWidth="1" style="39" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="42" t="inlineStr">
+        <is>
+          <t>Discretionary Spending Guardrail</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1" s="39">
+      <c r="A2" s="43" t="inlineStr">
+        <is>
+          <t>Three lanes — Matt, Sue, Household — for dinners, drinks, coffee, entertainment, convenience &amp; vices. Unused budget ROLLS OVER, so a high 'available' balance = green light to splurge; a negative one = pause. ORANGE = inputs (actuals arrive via Monthly Entry). Educational tool, not advice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="44" t="inlineStr">
+        <is>
+          <t>① BUDGET CONFIG  (per month)</t>
+        </is>
+      </c>
+      <c r="B4" s="45" t="n"/>
+      <c r="C4" s="45" t="n"/>
+      <c r="D4" s="45" t="n"/>
+      <c r="E4" s="45" t="n"/>
+      <c r="F4" s="45" t="n"/>
+      <c r="G4" s="45" t="n"/>
+      <c r="H4" s="45" t="n"/>
+      <c r="I4" s="45" t="n"/>
+      <c r="J4" s="45" t="n"/>
+      <c r="K4" s="45" t="n"/>
+      <c r="L4" s="45" t="n"/>
+      <c r="M4" s="45" t="n"/>
+      <c r="N4" s="45" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Matt monthly budget</t>
+        </is>
+      </c>
+      <c r="B5" s="50" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Sue monthly budget</t>
+        </is>
+      </c>
+      <c r="B6" s="50" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Household monthly budget</t>
+        </is>
+      </c>
+      <c r="B7" s="50" t="n">
+        <v>300</v>
+      </c>
+      <c r="C7" s="47" t="inlineStr">
+        <is>
+          <t>Shared dinners/entertainment together — set to taste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="63" t="inlineStr">
+        <is>
+          <t>Combined monthly budget</t>
+        </is>
+      </c>
+      <c r="B8" s="95">
+        <f>B5+B6+B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Splurge-room threshold ($)</t>
+        </is>
+      </c>
+      <c r="B9" s="50" t="n">
+        <v>150</v>
+      </c>
+      <c r="C9" s="47" t="inlineStr">
+        <is>
+          <t>When a lane's rollover balance clears this, it's green to splurge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Reporting month</t>
+        </is>
+      </c>
+      <c r="B10" s="49" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="C10" s="47" t="inlineStr">
+        <is>
+          <t>Drives the standings panel below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="44" t="inlineStr">
+        <is>
+          <t>② WHERE YOU STAND  (reporting month)</t>
+        </is>
+      </c>
+      <c r="B12" s="45" t="n"/>
+      <c r="C12" s="45" t="n"/>
+      <c r="D12" s="45" t="n"/>
+      <c r="E12" s="45" t="n"/>
+      <c r="F12" s="45" t="n"/>
+      <c r="G12" s="45" t="n"/>
+      <c r="H12" s="45" t="n"/>
+      <c r="I12" s="45" t="n"/>
+      <c r="J12" s="45" t="n"/>
+      <c r="K12" s="45" t="n"/>
+      <c r="L12" s="45" t="n"/>
+      <c r="M12" s="45" t="n"/>
+      <c r="N12" s="45" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="53" t="inlineStr">
+        <is>
+          <t>Lane</t>
+        </is>
+      </c>
+      <c r="B13" s="53" t="inlineStr">
+        <is>
+          <t>Budget</t>
+        </is>
+      </c>
+      <c r="C13" s="53" t="inlineStr">
+        <is>
+          <t>Spent (mo)</t>
+        </is>
+      </c>
+      <c r="D13" s="53" t="inlineStr">
+        <is>
+          <t>Rollover avail.</t>
+        </is>
+      </c>
+      <c r="E13" s="53" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="83" t="inlineStr">
+        <is>
+          <t>Matt</t>
+        </is>
+      </c>
+      <c r="B14" s="68">
+        <f>B5</f>
+        <v/>
+      </c>
+      <c r="C14" s="68">
+        <f>INDEX(B22:M22,MATCH($B$10,{"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec"},0))</f>
+        <v/>
+      </c>
+      <c r="D14" s="82">
+        <f>INDEX(B23:M23,MATCH($B$10,{"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec"},0))</f>
+        <v/>
+      </c>
+      <c r="E14" s="83">
+        <f>IF(D14="","",IF(D14&lt;0,"🔴 over — pause",IF(D14&gt;=$B$9,"🟢 splurge OK","🟡 on track")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="83" t="inlineStr">
+        <is>
+          <t>Sue</t>
+        </is>
+      </c>
+      <c r="B15" s="68">
+        <f>B6</f>
+        <v/>
+      </c>
+      <c r="C15" s="68">
+        <f>INDEX(B25:M25,MATCH($B$10,{"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec"},0))</f>
+        <v/>
+      </c>
+      <c r="D15" s="82">
+        <f>INDEX(B26:M26,MATCH($B$10,{"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec"},0))</f>
+        <v/>
+      </c>
+      <c r="E15" s="83">
+        <f>IF(D15="","",IF(D15&lt;0,"🔴 over — pause",IF(D15&gt;=$B$9,"🟢 splurge OK","🟡 on track")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="83" t="inlineStr">
+        <is>
+          <t>Household</t>
+        </is>
+      </c>
+      <c r="B16" s="68">
+        <f>B7</f>
+        <v/>
+      </c>
+      <c r="C16" s="68">
+        <f>INDEX(B28:M28,MATCH($B$10,{"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec"},0))</f>
+        <v/>
+      </c>
+      <c r="D16" s="82">
+        <f>INDEX(B29:M29,MATCH($B$10,{"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec"},0))</f>
+        <v/>
+      </c>
+      <c r="E16" s="83">
+        <f>IF(D16="","",IF(D16&lt;0,"🔴 over — pause",IF(D16&gt;=$B$9,"🟢 splurge OK","🟡 on track")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="80" t="inlineStr">
+        <is>
+          <t>Combined</t>
+        </is>
+      </c>
+      <c r="B17" s="68">
+        <f>B8</f>
+        <v/>
+      </c>
+      <c r="C17" s="68">
+        <f>INDEX(B30:M30,MATCH($B$10,{"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec"},0))</f>
+        <v/>
+      </c>
+      <c r="D17" s="82">
+        <f>INDEX(B32:M32,MATCH($B$10,{"Jan","Feb","Mar","Apr","May","Jun","Jul","Aug","Sep","Oct","Nov","Dec"},0))</f>
+        <v/>
+      </c>
+      <c r="E17" s="83">
+        <f>IF(D17="","",IF(D17&lt;0,"🔴 over — pause",IF(D17&gt;=$B$9,"🟢 splurge OK","🟡 on track")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="44" t="inlineStr">
+        <is>
+          <t>③ MONTHLY TRACKER  (rollover carries forward)</t>
+        </is>
+      </c>
+      <c r="B19" s="45" t="n"/>
+      <c r="C19" s="45" t="n"/>
+      <c r="D19" s="45" t="n"/>
+      <c r="E19" s="45" t="n"/>
+      <c r="F19" s="45" t="n"/>
+      <c r="G19" s="45" t="n"/>
+      <c r="H19" s="45" t="n"/>
+      <c r="I19" s="45" t="n"/>
+      <c r="J19" s="45" t="n"/>
+      <c r="K19" s="45" t="n"/>
+      <c r="L19" s="45" t="n"/>
+      <c r="M19" s="45" t="n"/>
+      <c r="N19" s="45" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="96" t="inlineStr"/>
+      <c r="B20" s="53" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="C20" s="53" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="D20" s="53" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="E20" s="53" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="F20" s="53" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="G20" s="53" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="H20" s="53" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="I20" s="53" t="inlineStr">
+        <is>
+          <t>Aug</t>
+        </is>
+      </c>
+      <c r="J20" s="53" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="K20" s="53" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="L20" s="53" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="M20" s="53" t="inlineStr">
+        <is>
+          <t>Dec</t>
+        </is>
+      </c>
+      <c r="N20" s="53" t="inlineStr">
+        <is>
+          <t>YTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="83" t="inlineStr">
+        <is>
+          <t>Matt — Budget</t>
+        </is>
+      </c>
+      <c r="B21" s="68">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="C21" s="68">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="D21" s="68">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="E21" s="68">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="F21" s="68">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="G21" s="68">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="H21" s="68">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="I21" s="68">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="J21" s="68">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="K21" s="68">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="L21" s="68">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="M21" s="68">
+        <f>$B$5</f>
+        <v/>
+      </c>
+      <c r="N21" s="68">
+        <f>SUM(B21:M21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="83" t="inlineStr">
+        <is>
+          <t>Matt — Actual (spent)</t>
+        </is>
+      </c>
+      <c r="B22" s="84" t="n"/>
+      <c r="C22" s="84" t="n"/>
+      <c r="D22" s="84" t="n"/>
+      <c r="E22" s="84" t="n"/>
+      <c r="F22" s="84" t="n"/>
+      <c r="G22" s="84" t="n"/>
+      <c r="H22" s="84" t="n"/>
+      <c r="I22" s="84" t="n"/>
+      <c r="J22" s="84" t="n"/>
+      <c r="K22" s="84" t="n"/>
+      <c r="L22" s="84" t="n"/>
+      <c r="M22" s="84" t="n"/>
+      <c r="N22" s="68">
+        <f>SUM(B22:M22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="80" t="inlineStr">
+        <is>
+          <t>Matt — Rollover available</t>
+        </is>
+      </c>
+      <c r="B23" s="85">
+        <f>B21-B22</f>
+        <v/>
+      </c>
+      <c r="C23" s="85">
+        <f>B23+C21-C22</f>
+        <v/>
+      </c>
+      <c r="D23" s="85">
+        <f>C23+D21-D22</f>
+        <v/>
+      </c>
+      <c r="E23" s="85">
+        <f>D23+E21-E22</f>
+        <v/>
+      </c>
+      <c r="F23" s="85">
+        <f>E23+F21-F22</f>
+        <v/>
+      </c>
+      <c r="G23" s="85">
+        <f>F23+G21-G22</f>
+        <v/>
+      </c>
+      <c r="H23" s="85">
+        <f>G23+H21-H22</f>
+        <v/>
+      </c>
+      <c r="I23" s="85">
+        <f>H23+I21-I22</f>
+        <v/>
+      </c>
+      <c r="J23" s="85">
+        <f>I23+J21-J22</f>
+        <v/>
+      </c>
+      <c r="K23" s="85">
+        <f>J23+K21-K22</f>
+        <v/>
+      </c>
+      <c r="L23" s="85">
+        <f>K23+L21-L22</f>
+        <v/>
+      </c>
+      <c r="M23" s="85">
+        <f>L23+M21-M22</f>
+        <v/>
+      </c>
+      <c r="N23" s="85">
+        <f>M23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="83" t="inlineStr">
+        <is>
+          <t>Sue — Budget</t>
+        </is>
+      </c>
+      <c r="B24" s="68">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="C24" s="68">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="D24" s="68">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="E24" s="68">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="F24" s="68">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="G24" s="68">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="H24" s="68">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="I24" s="68">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="J24" s="68">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="K24" s="68">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="L24" s="68">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="M24" s="68">
+        <f>$B$6</f>
+        <v/>
+      </c>
+      <c r="N24" s="68">
+        <f>SUM(B24:M24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="83" t="inlineStr">
+        <is>
+          <t>Sue — Actual (spent)</t>
+        </is>
+      </c>
+      <c r="B25" s="84" t="n"/>
+      <c r="C25" s="84" t="n"/>
+      <c r="D25" s="84" t="n"/>
+      <c r="E25" s="84" t="n"/>
+      <c r="F25" s="84" t="n"/>
+      <c r="G25" s="84" t="n"/>
+      <c r="H25" s="84" t="n"/>
+      <c r="I25" s="84" t="n"/>
+      <c r="J25" s="84" t="n"/>
+      <c r="K25" s="84" t="n"/>
+      <c r="L25" s="84" t="n"/>
+      <c r="M25" s="84" t="n"/>
+      <c r="N25" s="68">
+        <f>SUM(B25:M25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="80" t="inlineStr">
+        <is>
+          <t>Sue — Rollover available</t>
+        </is>
+      </c>
+      <c r="B26" s="85">
+        <f>B24-B25</f>
+        <v/>
+      </c>
+      <c r="C26" s="85">
+        <f>B26+C24-C25</f>
+        <v/>
+      </c>
+      <c r="D26" s="85">
+        <f>C26+D24-D25</f>
+        <v/>
+      </c>
+      <c r="E26" s="85">
+        <f>D26+E24-E25</f>
+        <v/>
+      </c>
+      <c r="F26" s="85">
+        <f>E26+F24-F25</f>
+        <v/>
+      </c>
+      <c r="G26" s="85">
+        <f>F26+G24-G25</f>
+        <v/>
+      </c>
+      <c r="H26" s="85">
+        <f>G26+H24-H25</f>
+        <v/>
+      </c>
+      <c r="I26" s="85">
+        <f>H26+I24-I25</f>
+        <v/>
+      </c>
+      <c r="J26" s="85">
+        <f>I26+J24-J25</f>
+        <v/>
+      </c>
+      <c r="K26" s="85">
+        <f>J26+K24-K25</f>
+        <v/>
+      </c>
+      <c r="L26" s="85">
+        <f>K26+L24-L25</f>
+        <v/>
+      </c>
+      <c r="M26" s="85">
+        <f>L26+M24-M25</f>
+        <v/>
+      </c>
+      <c r="N26" s="85">
+        <f>M26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="83" t="inlineStr">
+        <is>
+          <t>Household — Budget</t>
+        </is>
+      </c>
+      <c r="B27" s="68">
+        <f>$B$7</f>
+        <v/>
+      </c>
+      <c r="C27" s="68">
+        <f>$B$7</f>
+        <v/>
+      </c>
+      <c r="D27" s="68">
+        <f>$B$7</f>
+        <v/>
+      </c>
+      <c r="E27" s="68">
+        <f>$B$7</f>
+        <v/>
+      </c>
+      <c r="F27" s="68">
+        <f>$B$7</f>
+        <v/>
+      </c>
+      <c r="G27" s="68">
+        <f>$B$7</f>
+        <v/>
+      </c>
+      <c r="H27" s="68">
+        <f>$B$7</f>
+        <v/>
+      </c>
+      <c r="I27" s="68">
+        <f>$B$7</f>
+        <v/>
+      </c>
+      <c r="J27" s="68">
+        <f>$B$7</f>
+        <v/>
+      </c>
+      <c r="K27" s="68">
+        <f>$B$7</f>
+        <v/>
+      </c>
+      <c r="L27" s="68">
+        <f>$B$7</f>
+        <v/>
+      </c>
+      <c r="M27" s="68">
+        <f>$B$7</f>
+        <v/>
+      </c>
+      <c r="N27" s="68">
+        <f>SUM(B27:M27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="83" t="inlineStr">
+        <is>
+          <t>Household — Actual (spent)</t>
+        </is>
+      </c>
+      <c r="B28" s="84" t="n"/>
+      <c r="C28" s="84" t="n"/>
+      <c r="D28" s="84" t="n"/>
+      <c r="E28" s="84" t="n"/>
+      <c r="F28" s="84" t="n"/>
+      <c r="G28" s="84" t="n"/>
+      <c r="H28" s="84" t="n"/>
+      <c r="I28" s="84" t="n"/>
+      <c r="J28" s="84" t="n"/>
+      <c r="K28" s="84" t="n"/>
+      <c r="L28" s="84" t="n"/>
+      <c r="M28" s="84" t="n"/>
+      <c r="N28" s="68">
+        <f>SUM(B28:M28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="80" t="inlineStr">
+        <is>
+          <t>Household — Rollover available</t>
+        </is>
+      </c>
+      <c r="B29" s="85">
+        <f>B27-B28</f>
+        <v/>
+      </c>
+      <c r="C29" s="85">
+        <f>B29+C27-C28</f>
+        <v/>
+      </c>
+      <c r="D29" s="85">
+        <f>C29+D27-D28</f>
+        <v/>
+      </c>
+      <c r="E29" s="85">
+        <f>D29+E27-E28</f>
+        <v/>
+      </c>
+      <c r="F29" s="85">
+        <f>E29+F27-F28</f>
+        <v/>
+      </c>
+      <c r="G29" s="85">
+        <f>F29+G27-G28</f>
+        <v/>
+      </c>
+      <c r="H29" s="85">
+        <f>G29+H27-H28</f>
+        <v/>
+      </c>
+      <c r="I29" s="85">
+        <f>H29+I27-I28</f>
+        <v/>
+      </c>
+      <c r="J29" s="85">
+        <f>I29+J27-J28</f>
+        <v/>
+      </c>
+      <c r="K29" s="85">
+        <f>J29+K27-K28</f>
+        <v/>
+      </c>
+      <c r="L29" s="85">
+        <f>K29+L27-L28</f>
+        <v/>
+      </c>
+      <c r="M29" s="85">
+        <f>L29+M27-M28</f>
+        <v/>
+      </c>
+      <c r="N29" s="85">
+        <f>M29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="83" t="inlineStr">
+        <is>
+          <t>Combined — Actual</t>
+        </is>
+      </c>
+      <c r="B30" s="68">
+        <f>B22+B25+B28</f>
+        <v/>
+      </c>
+      <c r="C30" s="68">
+        <f>C22+C25+C28</f>
+        <v/>
+      </c>
+      <c r="D30" s="68">
+        <f>D22+D25+D28</f>
+        <v/>
+      </c>
+      <c r="E30" s="68">
+        <f>E22+E25+E28</f>
+        <v/>
+      </c>
+      <c r="F30" s="68">
+        <f>F22+F25+F28</f>
+        <v/>
+      </c>
+      <c r="G30" s="68">
+        <f>G22+G25+G28</f>
+        <v/>
+      </c>
+      <c r="H30" s="68">
+        <f>H22+H25+H28</f>
+        <v/>
+      </c>
+      <c r="I30" s="68">
+        <f>I22+I25+I28</f>
+        <v/>
+      </c>
+      <c r="J30" s="68">
+        <f>J22+J25+J28</f>
+        <v/>
+      </c>
+      <c r="K30" s="68">
+        <f>K22+K25+K28</f>
+        <v/>
+      </c>
+      <c r="L30" s="68">
+        <f>L22+L25+L28</f>
+        <v/>
+      </c>
+      <c r="M30" s="68">
+        <f>M22+M25+M28</f>
+        <v/>
+      </c>
+      <c r="N30" s="68">
+        <f>SUM(B30:M30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="83" t="inlineStr">
+        <is>
+          <t>Combined — Budget</t>
+        </is>
+      </c>
+      <c r="B31" s="68">
+        <f>B21+B24+B27</f>
+        <v/>
+      </c>
+      <c r="C31" s="68">
+        <f>C21+C24+C27</f>
+        <v/>
+      </c>
+      <c r="D31" s="68">
+        <f>D21+D24+D27</f>
+        <v/>
+      </c>
+      <c r="E31" s="68">
+        <f>E21+E24+E27</f>
+        <v/>
+      </c>
+      <c r="F31" s="68">
+        <f>F21+F24+F27</f>
+        <v/>
+      </c>
+      <c r="G31" s="68">
+        <f>G21+G24+G27</f>
+        <v/>
+      </c>
+      <c r="H31" s="68">
+        <f>H21+H24+H27</f>
+        <v/>
+      </c>
+      <c r="I31" s="68">
+        <f>I21+I24+I27</f>
+        <v/>
+      </c>
+      <c r="J31" s="68">
+        <f>J21+J24+J27</f>
+        <v/>
+      </c>
+      <c r="K31" s="68">
+        <f>K21+K24+K27</f>
+        <v/>
+      </c>
+      <c r="L31" s="68">
+        <f>L21+L24+L27</f>
+        <v/>
+      </c>
+      <c r="M31" s="68">
+        <f>M21+M24+M27</f>
+        <v/>
+      </c>
+      <c r="N31" s="68">
+        <f>SUM(B31:M31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="80" t="inlineStr">
+        <is>
+          <t>Combined — Rollover available</t>
+        </is>
+      </c>
+      <c r="B32" s="85">
+        <f>B23+B26+B29</f>
+        <v/>
+      </c>
+      <c r="C32" s="85">
+        <f>C23+C26+C29</f>
+        <v/>
+      </c>
+      <c r="D32" s="85">
+        <f>D23+D26+D29</f>
+        <v/>
+      </c>
+      <c r="E32" s="85">
+        <f>E23+E26+E29</f>
+        <v/>
+      </c>
+      <c r="F32" s="85">
+        <f>F23+F26+F29</f>
+        <v/>
+      </c>
+      <c r="G32" s="85">
+        <f>G23+G26+G29</f>
+        <v/>
+      </c>
+      <c r="H32" s="85">
+        <f>H23+H26+H29</f>
+        <v/>
+      </c>
+      <c r="I32" s="85">
+        <f>I23+I26+I29</f>
+        <v/>
+      </c>
+      <c r="J32" s="85">
+        <f>J23+J26+J29</f>
+        <v/>
+      </c>
+      <c r="K32" s="85">
+        <f>K23+K26+K29</f>
+        <v/>
+      </c>
+      <c r="L32" s="85">
+        <f>L23+L26+L29</f>
+        <v/>
+      </c>
+      <c r="M32" s="85">
+        <f>M23+M26+M29</f>
+        <v/>
+      </c>
+      <c r="N32" s="85">
+        <f>M32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="44" t="inlineStr">
+        <is>
+          <t>④ IMPACT ON YOUR SAVINGS / FIRE</t>
+        </is>
+      </c>
+      <c r="B34" s="45" t="n"/>
+      <c r="C34" s="45" t="n"/>
+      <c r="D34" s="45" t="n"/>
+      <c r="E34" s="45" t="n"/>
+      <c r="F34" s="45" t="n"/>
+      <c r="G34" s="45" t="n"/>
+      <c r="H34" s="45" t="n"/>
+      <c r="I34" s="45" t="n"/>
+      <c r="J34" s="45" t="n"/>
+      <c r="K34" s="45" t="n"/>
+      <c r="L34" s="45" t="n"/>
+      <c r="M34" s="45" t="n"/>
+      <c r="N34" s="45" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>YTD combined budget</t>
+        </is>
+      </c>
+      <c r="B35" s="73">
+        <f>N31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>YTD combined actual</t>
+        </is>
+      </c>
+      <c r="B36" s="73">
+        <f>N30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="63" t="inlineStr">
+        <is>
+          <t>YTD over / (under)</t>
+        </is>
+      </c>
+      <c r="B37" s="64">
+        <f>N30-N31</f>
+        <v/>
+      </c>
+      <c r="C37" s="47" t="inlineStr">
+        <is>
+          <t>Positive = overspent (money that didn't get invested).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Growth factor (real, 20 yrs)</t>
+        </is>
+      </c>
+      <c r="B38" s="97">
+        <f>(1+'FIRE Dashboard'!B12)^20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="63" t="inlineStr">
+        <is>
+          <t>Compounded cost of overspend</t>
+        </is>
+      </c>
+      <c r="B39" s="64">
+        <f>MAX(0,B37)*B38</f>
+        <v/>
+      </c>
+      <c r="C39" s="47" t="inlineStr">
+        <is>
+          <t>What this year's overspend would be worth in 20 yrs if invested instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="41" t="inlineStr">
+        <is>
+          <t>How rollover works: each month adds the lane's budget and subtracts what you spent. Underspend and the balance grows (bank it for a guilt-free splurge later); overspend and it goes negative until you claw it back. Actuals post automatically from the Monthly Entry tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42"/>
+    <row r="43"/>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="C10:H10"/>
+    <mergeCell ref="C37:H37"/>
+    <mergeCell ref="C9:H9"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="C39:H39"/>
+    <mergeCell ref="A41:N43"/>
+    <mergeCell ref="C7:H7"/>
+  </mergeCells>
+  <conditionalFormatting sqref="B23:M23">
+    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="greaterThanOrEqual" dxfId="3">
+      <formula>$B$9</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B26:M26">
+    <cfRule type="cellIs" priority="3" operator="lessThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="greaterThanOrEqual" dxfId="3">
+      <formula>$B$9</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B29:M29">
+    <cfRule type="cellIs" priority="5" operator="lessThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="greaterThanOrEqual" dxfId="3">
+      <formula>$B$9</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B32:M32">
+    <cfRule type="cellIs" priority="7" operator="lessThan" dxfId="2">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" dxfId="3">
+      <formula>$B$9</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Jan,Feb,Mar,Apr,May,Jun,Jul,Aug,Sep,Oct,Nov,Dec"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Set Sue MTRS membership to 2010; pre-fill March solar from Enphase report
- Pension - Sue: effective membership date = 2010 (refund taken on 2003-07
  service, rejoined 2010); still Tier 1 + mandatory RetirementPlus, ~16 yrs
  creditable service (2010->2026).
- Solar Reinvestment: seeded March energy log from the Enphase monthly report
  (Produced 133.1, Consumed 661.4, Imported 528.3, Exported 0.0 kWh) as a
  worked example; updated the note to reflect seasonal production swings.
</commit_message>
<xml_diff>
--- a/Family_Income_Statement_2026_v5_FIRE.xlsx
+++ b/Family_Income_Statement_2026_v5_FIRE.xlsx
@@ -13901,11 +13901,11 @@
         </is>
       </c>
       <c r="B5" s="46" t="n">
-        <v>2003</v>
+        <v>2010</v>
       </c>
       <c r="C5" s="47" t="inlineStr">
         <is>
-          <t>2003 if funds left on account; 2010 if she took a refund &amp; rejoined. Either way = Tier 1.</t>
+          <t>Confirmed 2010 (refund taken on 2003–07 service, rejoined 2010). Post-2001 join → Tier 1, mandatory R+.</t>
         </is>
       </c>
     </row>
@@ -13920,7 +13920,7 @@
       </c>
       <c r="C6" s="47" t="inlineStr">
         <is>
-          <t>~16 if she refunded the 2003–07 years; ~20 if that service is still on account. MyTRS shows the exact figure.</t>
+          <t>~16 years (2010 → 2026, continuous). Confirm the exact figure in MyTRS.</t>
         </is>
       </c>
     </row>
@@ -16751,10 +16751,18 @@
           <t>Mar</t>
         </is>
       </c>
-      <c r="B16" s="86" t="n"/>
-      <c r="C16" s="86" t="n"/>
-      <c r="D16" s="86" t="n"/>
-      <c r="E16" s="86" t="n"/>
+      <c r="B16" s="86" t="n">
+        <v>133.1</v>
+      </c>
+      <c r="C16" s="86" t="n">
+        <v>661.4</v>
+      </c>
+      <c r="D16" s="86" t="n">
+        <v>528.3</v>
+      </c>
+      <c r="E16" s="86" t="n">
+        <v>0</v>
+      </c>
       <c r="F16" s="87">
         <f>E16-D16</f>
         <v/>
@@ -16925,7 +16933,7 @@
     <row r="27">
       <c r="A27" s="41" t="inlineStr">
         <is>
-          <t>Latest Enphase snapshot (dashboard view): Produced 3.4 MWh · Consumed 2.6 MWh · Imported 1.3 MWh · Exported 2.2 MWh · Net exported ~872 kWh · Solar offset 134%. Replace with monthly report values above.</t>
+          <t>Enter each month from your Enphase monthly report (no CSV export — read the tile values). Production swings seasonally: March is pre-filled from your report (133 kWh produced vs 661 consumed → net import), while summer months over-produce and export. Net export = Exported − Imported (negative = net import).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Seed May-August solar energy log from Enphase reports; refine production estimate
- Solar Reinvestment energy log: entered May, June, July, August from the
  monthly Enphase reports (April left blank - report not provided).
  June/July 'Produced' derived from the energy identity since the tiles
  rounded to 1.1 MWh. All readings reconcile (Produced = Consumed - Imported
  + Exported).
- Lowered est. annual production default to 7,000 kWh to match the 2026
  YTD trajectory (~5 MWh by August).
</commit_message>
<xml_diff>
--- a/Family_Income_Statement_2026_v5_FIRE.xlsx
+++ b/Family_Income_Statement_2026_v5_FIRE.xlsx
@@ -16789,10 +16789,18 @@
           <t>May</t>
         </is>
       </c>
-      <c r="B18" s="86" t="n"/>
-      <c r="C18" s="86" t="n"/>
-      <c r="D18" s="86" t="n"/>
-      <c r="E18" s="86" t="n"/>
+      <c r="B18" s="86" t="n">
+        <v>997.1</v>
+      </c>
+      <c r="C18" s="86" t="n">
+        <v>475.1</v>
+      </c>
+      <c r="D18" s="86" t="n">
+        <v>246.7</v>
+      </c>
+      <c r="E18" s="86" t="n">
+        <v>768.7</v>
+      </c>
       <c r="F18" s="87">
         <f>E18-D18</f>
         <v/>
@@ -16804,10 +16812,18 @@
           <t>Jun</t>
         </is>
       </c>
-      <c r="B19" s="86" t="n"/>
-      <c r="C19" s="86" t="n"/>
-      <c r="D19" s="86" t="n"/>
-      <c r="E19" s="86" t="n"/>
+      <c r="B19" s="86" t="n">
+        <v>1128.1</v>
+      </c>
+      <c r="C19" s="86" t="n">
+        <v>784.5</v>
+      </c>
+      <c r="D19" s="86" t="n">
+        <v>383</v>
+      </c>
+      <c r="E19" s="86" t="n">
+        <v>726.6</v>
+      </c>
       <c r="F19" s="87">
         <f>E19-D19</f>
         <v/>
@@ -16819,10 +16835,18 @@
           <t>Jul</t>
         </is>
       </c>
-      <c r="B20" s="86" t="n"/>
-      <c r="C20" s="86" t="n"/>
-      <c r="D20" s="86" t="n"/>
-      <c r="E20" s="86" t="n"/>
+      <c r="B20" s="86" t="n">
+        <v>1058.5</v>
+      </c>
+      <c r="C20" s="86" t="n">
+        <v>964.6</v>
+      </c>
+      <c r="D20" s="86" t="n">
+        <v>507.4</v>
+      </c>
+      <c r="E20" s="86" t="n">
+        <v>601.3</v>
+      </c>
       <c r="F20" s="87">
         <f>E20-D20</f>
         <v/>
@@ -16834,10 +16858,18 @@
           <t>Aug</t>
         </is>
       </c>
-      <c r="B21" s="86" t="n"/>
-      <c r="C21" s="86" t="n"/>
-      <c r="D21" s="86" t="n"/>
-      <c r="E21" s="86" t="n"/>
+      <c r="B21" s="86" t="n">
+        <v>919.3</v>
+      </c>
+      <c r="C21" s="86" t="n">
+        <v>938.4</v>
+      </c>
+      <c r="D21" s="86" t="n">
+        <v>531.1</v>
+      </c>
+      <c r="E21" s="86" t="n">
+        <v>512</v>
+      </c>
       <c r="F21" s="87">
         <f>E21-D21</f>
         <v/>
@@ -17021,7 +17053,12 @@
         </is>
       </c>
       <c r="B36" s="91" t="n">
-        <v>11000</v>
+        <v>7000</v>
+      </c>
+      <c r="C36" s="47" t="inlineStr">
+        <is>
+          <t>Rough full-year estimate from your 2026 trajectory (YTD ~5 MWh by Aug). Refine after a full year.</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -18030,12 +18067,13 @@
     <row r="79"/>
     <row r="80"/>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A12:H12"/>
     <mergeCell ref="C6:H6"/>
     <mergeCell ref="C32:H32"/>
     <mergeCell ref="C38:H38"/>
     <mergeCell ref="C41:H41"/>
+    <mergeCell ref="C36:H36"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="C31:H31"/>
     <mergeCell ref="A78:H80"/>

</xml_diff>

<commit_message>
Seed April solar (system commissioned mid-April); completes Mar-Aug log
April Enphase report: Produced 314.2 / Consumed 102.6 / Imported 50.1 /
Exported 261.7 kWh. Weekly chart shows production only from ~Apr 15-28 and
unusually low consumption, indicating mid-April commissioning (consistent
with 2026 placed-in-service and $0 federal ITC).
</commit_message>
<xml_diff>
--- a/Family_Income_Statement_2026_v5_FIRE.xlsx
+++ b/Family_Income_Statement_2026_v5_FIRE.xlsx
@@ -16774,10 +16774,18 @@
           <t>Apr</t>
         </is>
       </c>
-      <c r="B17" s="86" t="n"/>
-      <c r="C17" s="86" t="n"/>
-      <c r="D17" s="86" t="n"/>
-      <c r="E17" s="86" t="n"/>
+      <c r="B17" s="86" t="n">
+        <v>314.2</v>
+      </c>
+      <c r="C17" s="86" t="n">
+        <v>102.6</v>
+      </c>
+      <c r="D17" s="86" t="n">
+        <v>50.1</v>
+      </c>
+      <c r="E17" s="86" t="n">
+        <v>261.7</v>
+      </c>
       <c r="F17" s="87">
         <f>E17-D17</f>
         <v/>

</xml_diff>